<commit_message>
Add attachments and update POD dates
Fix README activation path and add missing attachments and documents for containers. Added invoice and packing list files and referenced them from data/container_HTML/25_05.json. Updated 25_06.html to include attachments and corrected POD/consignee details, and updated 25_06.json to shift the POD date to 2026-02-26 and clear the operation/comment fields. Also touched containers_data.csv, etas (CSV/JSON) and input/Containers.xlsx to reflect related metadata updates.
</commit_message>
<xml_diff>
--- a/input/Containers.xlsx
+++ b/input/Containers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Overzichtslijsten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07245F7A-1A5C-45FD-B70A-884795C3835A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB32926-8191-44F3-9C33-CD29041D63CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,12 +87,6 @@
     <t>https://transtrack.magaya.net/TransTracking?ID=38049&amp;SH=e7d91f0e-2326-4ca6-ae43-eb9eaf6e8e1d&amp;LG=en&amp;XM=0</t>
   </si>
   <si>
-    <t>25#8</t>
-  </si>
-  <si>
-    <t>25#9</t>
-  </si>
-  <si>
     <t>25172</t>
   </si>
   <si>
@@ -112,6 +106,12 @@
   </si>
   <si>
     <t>https://transtrack.magaya.net/TransTracking?ID=38049&amp;SH=e25a08a2-185f-4e0c-ae71-d5a9b0295662&amp;LG=en&amp;XM=0</t>
+  </si>
+  <si>
+    <t>25#08</t>
+  </si>
+  <si>
+    <t>25#09</t>
   </si>
 </sst>
 </file>
@@ -121,7 +121,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -160,8 +160,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,6 +178,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,12 +195,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -221,8 +234,22 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Goed" xfId="3" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Ongeldig" xfId="2" builtinId="27"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -559,23 +586,23 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="15">
         <v>13923</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="17">
         <v>46062</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="18" t="s">
         <v>18</v>
       </c>
     </row>
@@ -590,13 +617,13 @@
         <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E5" s="7">
-        <v>46075</v>
+        <v>46076</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -610,38 +637,39 @@
         <v>17</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E6" s="7">
-        <v>46109</v>
+        <v>46122</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B7" s="11">
         <v>14170</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F7" s="13"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B8" s="11">
         <v>14175</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>